<commit_message>
Cierre de tareas finales del proyecto y preparación de la versión de entrega
- Finalización de la documentación pendiente del proyecto.
- Actualización y reorganización de los materiales de apoyo para la guía de usuario.
- Revisión final de la presentación del TFG.
- Resubida y actualización del fichero Zotero con las referencias bibliográficas empleadas.
- Corrección de incidencias detectadas en el flujo de recuento de votaciones.
- Ajuste de los procesos de descifrado y validación criptográfica de votos.
- Corrección de la visualización de resultados y candidatura ganadora en la interfaz de mesa electoral.
- Revisión general y estabilización de la aplicación previa a la generación de la versión final.

Closes #1
Closes #38
Closes #42
Closes #43
</commit_message>
<xml_diff>
--- a/media/Plantilla_Censos.xlsx
+++ b/media/Plantilla_Censos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alons\OneDrive\Escritorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alons\OneDrive\Escritorio\Televot_APP\TeleVotApp-2\media\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D696C8-3D97-4C4A-B6CB-BB37D5380394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9443731C-D9DD-42DB-92FD-22A7938F6D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3E07C450-C0F7-4214-8F6D-C999D9237F6C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E07C450-C0F7-4214-8F6D-C999D9237F6C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>DNI</t>
   </si>
@@ -48,126 +48,6 @@
   </si>
   <si>
     <t>Email</t>
-  </si>
-  <si>
-    <t>12345678A</t>
-  </si>
-  <si>
-    <t>Marta</t>
-  </si>
-  <si>
-    <t>Rodríguez López</t>
-  </si>
-  <si>
-    <t>marta.rodriguez@email.com</t>
-  </si>
-  <si>
-    <t>87654321B</t>
-  </si>
-  <si>
-    <t>Javier</t>
-  </si>
-  <si>
-    <t>García Fernández</t>
-  </si>
-  <si>
-    <t>j.garciafernandez@mail.es</t>
-  </si>
-  <si>
-    <t>23456789C</t>
-  </si>
-  <si>
-    <t>Lucía</t>
-  </si>
-  <si>
-    <t>Sánchez Martínez</t>
-  </si>
-  <si>
-    <t>lucia.sanchez90@gmail.com</t>
-  </si>
-  <si>
-    <t>34567890D</t>
-  </si>
-  <si>
-    <t>Álvaro</t>
-  </si>
-  <si>
-    <t>Pérez Gómez</t>
-  </si>
-  <si>
-    <t>alvaro.perez.gomez@outlook.com</t>
-  </si>
-  <si>
-    <t>45678901E</t>
-  </si>
-  <si>
-    <t>Carmen</t>
-  </si>
-  <si>
-    <t>Torres Ruiz</t>
-  </si>
-  <si>
-    <t>carmen.torres@mail.com</t>
-  </si>
-  <si>
-    <t>56789012F</t>
-  </si>
-  <si>
-    <t>Diego</t>
-  </si>
-  <si>
-    <t>Romero Ortega</t>
-  </si>
-  <si>
-    <t>diego.romero.93@gmail.com</t>
-  </si>
-  <si>
-    <t>67890123G</t>
-  </si>
-  <si>
-    <t>Elena</t>
-  </si>
-  <si>
-    <t>Morales Hidalgo</t>
-  </si>
-  <si>
-    <t>elena.mhidalgo@correo.es</t>
-  </si>
-  <si>
-    <t>78901234H</t>
-  </si>
-  <si>
-    <t>Sergio</t>
-  </si>
-  <si>
-    <t>Navarro León</t>
-  </si>
-  <si>
-    <t>s.navarro.leon@outlook.com</t>
-  </si>
-  <si>
-    <t>89012345J</t>
-  </si>
-  <si>
-    <t>Laura</t>
-  </si>
-  <si>
-    <t>Molina Serrano</t>
-  </si>
-  <si>
-    <t>laura.molina.s@gmail.com</t>
-  </si>
-  <si>
-    <t>90123456K</t>
-  </si>
-  <si>
-    <t>Andrés</t>
-  </si>
-  <si>
-    <t>Ibáñez Castillo</t>
-  </si>
-  <si>
-    <t>andres.icastillo@mail.com</t>
   </si>
 </sst>
 </file>
@@ -602,144 +482,64 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>31</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>39</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
@@ -916,18 +716,6 @@
       <c r="D40" s="1"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" display="mailto:marta.rodriguez@email.com" xr:uid="{14E5FB9C-1785-4FD1-9CD1-9DAB91043E82}"/>
-    <hyperlink ref="D3" r:id="rId2" display="mailto:j.garciafernandez@mail.es" xr:uid="{FDD2F7D5-C99A-43CE-84BB-763DCB624A47}"/>
-    <hyperlink ref="D4" r:id="rId3" display="mailto:lucia.sanchez90@gmail.com" xr:uid="{56552AFC-5C34-4482-893B-EC4D9DF19977}"/>
-    <hyperlink ref="D5" r:id="rId4" display="mailto:alvaro.perez.gomez@outlook.com" xr:uid="{101C0210-60A8-4E72-93DA-63E173346123}"/>
-    <hyperlink ref="D6" r:id="rId5" display="mailto:carmen.torres@mail.com" xr:uid="{C7192E48-515B-4B4D-B7A5-369F0C726744}"/>
-    <hyperlink ref="D7" r:id="rId6" display="mailto:diego.romero.93@gmail.com" xr:uid="{B7E8A01D-85D1-4182-965E-E94DDA3F46BF}"/>
-    <hyperlink ref="D8" r:id="rId7" display="mailto:elena.mhidalgo@correo.es" xr:uid="{A72431C9-69D1-4C24-A75B-DB55662123F6}"/>
-    <hyperlink ref="D9" r:id="rId8" display="mailto:s.navarro.leon@outlook.com" xr:uid="{AA68569D-E432-49A5-9E32-8AFA0790B54F}"/>
-    <hyperlink ref="D10" r:id="rId9" display="mailto:laura.molina.s@gmail.com" xr:uid="{68153EC6-C295-45B1-9688-5A23E95E1252}"/>
-    <hyperlink ref="D11" r:id="rId10" display="mailto:andres.icastillo@mail.com" xr:uid="{94B0CE60-DA4C-4953-8105-10171038A539}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>